<commit_message>
add google-genai dependency and update files
</commit_message>
<xml_diff>
--- a/my_projects.xlsx
+++ b/my_projects.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sivane\Desktop\ai-project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sivane\Desktop\ai-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C2009F-0D12-4414-955A-13FEDBDF539C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A13E75D-FF2A-4C84-9465-A587AB8BDB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{1968CE39-0EE5-4883-A237-EBC97DE891BE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
   <si>
     <t>project_name</t>
   </si>
@@ -60,6 +60,24 @@
   </si>
   <si>
     <t>אדום</t>
+  </si>
+  <si>
+    <t xml:space="preserve">דנאל </t>
+  </si>
+  <si>
+    <t>בנק יהב</t>
+  </si>
+  <si>
+    <t>project_type</t>
+  </si>
+  <si>
+    <t>פרויקט אקטיבי</t>
+  </si>
+  <si>
+    <t>חבילות עבודה</t>
+  </si>
+  <si>
+    <t>תחזוקה</t>
   </si>
 </sst>
 </file>
@@ -432,43 +450,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A4D3777-BE6E-4350-B7B6-59736C5B393D}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.58203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>